<commit_message>
Refresh (23 Oct 2026 run): add 10 live-exam notifications (APPSC, RRB Station Master, NTA CSIR-UGC NET & NIFTEE), fill AP detailed-notice age limits, add 3 career-magazine entries
</commit_message>
<xml_diff>
--- a/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
@@ -689,7 +689,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 22 October 2026 | updated 22 October 2026 with the 1-22 October 2026 scrape</t>
+          <t>Compiled 23 October 2026 | updated 23 October 2026 with the 1-23 October 2026 scrape</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Status is as of 22 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
+          <t>Status is as of 23 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
         </is>
       </c>
     </row>
@@ -821,8 +821,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B9:D10"/>
     <mergeCell ref="B11:D12"/>
-    <mergeCell ref="B9:D10"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
   </mergeCells>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -2987,417 +2987,591 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr"/>
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Naval Dockyard Mumbai Apprentice Recruitment 2026 (283 trade apprentices)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Naval Dockyard Mumbai (Indian Navy), Ministry of Defence</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>ITI candidates in designated trades (Electrician, Electronics Mechanic, Fitter, Machinist, Welder, Pipe Fitter, Turner, Shipwright and others) at the Naval Dockyard Apprentice School</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <t>As per trade norms</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="16" t="inlineStr">
         <is>
           <t>Annual (designated trades)</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="K26" s="16" t="inlineStr">
         <is>
           <t>Paid apprenticeship as per the Apprentices Act; 283 vacancies across designated trades (Electrician, Fitter, Machinist, Welder, etc.)</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="L26" s="16" t="inlineStr">
         <is>
           <t>Last date 27-Oct-2026</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="M26" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="N26" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="O26" s="16" t="inlineStr">
         <is>
           <t>www.employmentnews.gov.in</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="P26" s="16" t="inlineStr">
         <is>
           <t>https://www.indgovtjobs.in/2017/04/Employment-News.html</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q26" s="16" t="inlineStr">
         <is>
           <t>Appears in the Employment News 03-09 October 2026 issue (Pages 16-20)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr"/>
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Scholarship / Fellowship</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>CCRAS Fellowship 2026 (Research Fellowship)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Central Council for Research in Ayurvedic Sciences (CCRAS), Ministry of AYUSH</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Postgraduate / research candidates in Ayurvedic and allied sciences</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>As per fellowship norms</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>As per notification</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="16" t="inlineStr">
         <is>
           <t>Annual</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="K27" s="16" t="inlineStr">
         <is>
           <t>Research fellowship as per CCRAS norms; 25 posts</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="L27" s="16" t="inlineStr">
         <is>
           <t>Last date 08-Dec-2026</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="M27" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="N27" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="O27" s="16" t="inlineStr">
         <is>
           <t>www.ccras.nic.in</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="P27" s="16" t="inlineStr">
         <is>
           <t>https://www.indgovtjobs.in/2017/04/Employment-News.html</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" s="16" t="inlineStr">
         <is>
           <t>Listed in the Employment News 09-16 October 2026 issue</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr"/>
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Scholarship / Fellowship</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>NTA CSIR-UGC NET December 2026 (JRF &amp; Assistant Professor eligibility)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>National Testing Agency (NTA) on behalf of CSIR</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Postgraduate science candidates (M.Sc or equivalent) for JRF and Assistant Professor eligibility</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <t>As per CSIR-UGC NET norms (upper age for JRF)</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="16" t="inlineStr">
         <is>
           <t>Twice-yearly</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>Junior Research Fellowship and Assistant Professor eligibility; exam fee as per NTA</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L28" s="16" t="inlineStr">
         <is>
           <t>Last date 05-Nov-2026</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M28" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="N28" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="O28" s="16" t="inlineStr">
         <is>
           <t>https://csirnet.nta.ac.in</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="P28" s="16" t="inlineStr">
         <is>
           <t>https://www.indgovtjobs.in/2017/04/Employment-News.html</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="Q28" s="16" t="inlineStr">
         <is>
           <t>Listed in the Employment News 17-23 October 2026 issue</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr"/>
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>ICAR-IARI Young Professionals 2026 (4 posts)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="16" t="inlineStr">
         <is>
           <t>ICAR - Indian Agricultural Research Institute (IARI)</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Graduate / postgraduate candidates for project-based Young Professional positions</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>As per ICAR norms</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>As per notification</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="16" t="inlineStr">
         <is>
           <t>Contractual (project-based)</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K29" s="16" t="inlineStr">
         <is>
           <t>Young Professional honorarium as per ICAR norms; 4 posts</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L29" s="16" t="inlineStr">
         <is>
           <t>Last date 25-Oct-2026</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M29" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="N29" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="O29" s="16" t="inlineStr">
         <is>
           <t>https://www.iari.res.in</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="P29" s="16" t="inlineStr">
         <is>
           <t>https://www.indgovtjobs.in/2017/04/Employment-News.html</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="Q29" s="16" t="inlineStr">
         <is>
           <t>Listed in the Employment News 17-23 October 2026 issue</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>Scholarship / Fellowship</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>DBT-BET Junior Research Fellowship (DBT-JRF) 2026-27</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>Department of Biotechnology (DBT), Ministry of Science &amp; Technology</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Postgraduate candidates in biotechnology and allied life-science subjects (via the DBT-BET examination)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="16" t="inlineStr">
         <is>
           <t>As per DBT-BET norms</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="16" t="inlineStr">
         <is>
           <t>Annual</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="K30" s="16" t="inlineStr">
         <is>
           <t>Junior Research Fellowship (approx Rs 37,000 per month plus HRA) for the fellowship tenure</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="L30" s="16" t="inlineStr">
         <is>
           <t>Last date 15-Nov-2026</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M30" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N30" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="O30" s="16" t="inlineStr">
         <is>
           <t>https://dbt.nta.ac.in</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="P30" s="16" t="inlineStr">
         <is>
           <t>https://www.indiascholarships.in/scholarships/recently-added</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="Q30" s="16" t="inlineStr">
         <is>
           <t>Listed among scholarships closing in Nov 2026 (Employment News / aggregator round-ups)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>Scholarship / Fellowship</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>IndiaAI Fellowship 2026 (UG, PG and PhD students)</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Ministry of Electronics and Information Technology (MeitY), Government of India</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Undergraduate, postgraduate and PhD students working in Artificial Intelligence and allied areas</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Open to all</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>As per scheme norms</t>
+        </is>
+      </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>Annual (2026 call)</t>
+        </is>
+      </c>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>Financial support of up to Rs.1,00,000 for UG students and up to Rs.2,00,000 for PG students (as announced by MeitY)</t>
+        </is>
+      </c>
+      <c r="L31" s="16" t="inlineStr">
+        <is>
+          <t>Last date 30-11-2026</t>
+        </is>
+      </c>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="N31" s="16" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O31" s="16" t="inlineStr">
+        <is>
+          <t>indiaai.gov.in</t>
+        </is>
+      </c>
+      <c r="P31" s="16" t="inlineStr">
+        <is>
+          <t>https://indianexpress.com/article/education/meity-indiaai-offers-fellowship-with-financial-support-up-to-rs-1-lakh-for-ug-students-rs-2-lakh-for-pg-students-govt-10930508/</t>
+        </is>
+      </c>
+      <c r="Q31" s="16" t="inlineStr">
+        <is>
+          <t>IndiaAI Fellowship announced by MeitY (October 2026), applications close 30 November 2026. Included as upcoming Employment News coverage of a central-government fellowship; the specific EN issue placement was not directly verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>NIFT Entrance Examination (NIFTEE) 2027 - UG, PG, NLEA, Artisans and PhD programmes</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>National Testing Agency (NTA) on behalf of the National Institute of Fashion Technology (NIFT)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Class 12 students (UG), graduates (PG) and others as per programme</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>As per programme norms</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Annual (2027 admission cycle)</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Admission to NIFT UG / PG / NLEA / Artisans / PhD programmes; exam fee as per the NTA information bulletin</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>As per the NTA information bulletin</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>nift.ac.in</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>https://nta.ac.in/NoticeBoardArchive</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>NTA has invited online applications for NIFTEE-2027 (NTA notice board, October 2026). Included as upcoming Employment News coverage of an NTA entrance exam; the specific EN issue placement was not directly verified.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh: live exam notifications (71) + career magazines (205) - 24 Oct 2026
</commit_message>
<xml_diff>
--- a/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
@@ -689,7 +689,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 23 October 2026 | updated 23 October 2026 with the 1-23 October 2026 scrape</t>
+          <t>Compiled 24 October 2026 | updated 24 October 2026 with the 1-24 October 2026 scrape</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Status is as of 23 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
+          <t>Status is as of 24 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
         </is>
       </c>
     </row>
@@ -821,8 +821,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B9:D10"/>
-    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
   </mergeCells>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -3489,89 +3489,176 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>Admission / Entrance Exam</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>NIFT Entrance Examination (NIFTEE) 2027 - UG, PG, NLEA, Artisans and PhD programmes</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>National Testing Agency (NTA) on behalf of the National Institute of Fashion Technology (NIFT)</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>Class 12 students (UG), graduates (PG) and others as per programme</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="16" t="inlineStr">
         <is>
           <t>As per programme norms</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="16" t="inlineStr">
         <is>
           <t>Annual (2027 admission cycle)</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K32" s="16" t="inlineStr">
         <is>
           <t>Admission to NIFT UG / PG / NLEA / Artisans / PhD programmes; exam fee as per the NTA information bulletin</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L32" s="16" t="inlineStr">
         <is>
           <t>As per the NTA information bulletin</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N32" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="O32" s="16" t="inlineStr">
         <is>
           <t>nift.ac.in</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="P32" s="16" t="inlineStr">
         <is>
           <t>https://nta.ac.in/NoticeBoardArchive</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="Q32" s="16" t="inlineStr">
         <is>
           <t>NTA has invited online applications for NIFTEE-2027 (NTA notice board, October 2026). Included as upcoming Employment News coverage of an NTA entrance exam; the specific EN issue placement was not directly verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Scholarship / Fellowship</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Swami Dayanand Education Foundation (SDEF) Scholarship 2026-27</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Swami Dayanand Education Foundation (SDEF), New Delhi</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>First-year students of professional courses (engineering, medical, law, management) and open-degree courses at recognised Indian institutions</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>All categories (means-based)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Means-based; SDEF family-income criteria apply</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>As per notification</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Annual (2026-27)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Up to Rs.50,000 per year towards tuition and fees (means-based); number of awards as per SDEF</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Last date 31-10-2026</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>https://www.swamidayanand.org</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>https://www.inextlive.com/top-scholarships-and-internships-to-apply-for-in-october-2026-1791380527</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Means-based scholarship for first-year professional/open-degree students, 2026-27 cycle (applications close 31 October 2026). Included as Employment News-type central scholarship coverage; the specific EN issue placement was not directly verified.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh opportunity tracker (25 Oct 2026 run)
</commit_message>
<xml_diff>
--- a/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
@@ -689,7 +689,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 24 October 2026 | updated 24 October 2026 with the 1-24 October 2026 scrape</t>
+          <t>Compiled 25 October 2026 | updated 25 October 2026 with the 1-25 October 2026 scrape</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Status is as of 24 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
+          <t>Status is as of 25 October 2026: green = open now, blue = rolling applications, amber = upcoming, grey = dates to be announced, red = closed. Closed items are retained because most exams and scholarship cycles are annual and repeat each year.</t>
         </is>
       </c>
     </row>
@@ -821,10 +821,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B9:D10"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
+    <mergeCell ref="B11:D12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -3576,89 +3576,344 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>Scholarship / Fellowship</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
         <is>
           <t>Swami Dayanand Education Foundation (SDEF) Scholarship 2026-27</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>Swami Dayanand Education Foundation (SDEF), New Delhi</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="16" t="inlineStr">
         <is>
           <t>First-year students of professional courses (engineering, medical, law, management) and open-degree courses at recognised Indian institutions</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="16" t="inlineStr">
         <is>
           <t>All categories (means-based)</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="16" t="inlineStr">
         <is>
           <t>Means-based; SDEF family-income criteria apply</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="16" t="inlineStr">
         <is>
           <t>As per notification</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="16" t="inlineStr">
         <is>
           <t>Annual (2026-27)</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="16" t="inlineStr">
         <is>
           <t>Up to Rs.50,000 per year towards tuition and fees (means-based); number of awards as per SDEF</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="L33" s="16" t="inlineStr">
         <is>
           <t>Last date 31-10-2026</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="M33" s="16" t="inlineStr">
         <is>
           <t>Open now</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="N33" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="O33" s="16" t="inlineStr">
         <is>
           <t>https://www.swamidayanand.org</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" s="16" t="inlineStr">
         <is>
           <t>https://www.inextlive.com/top-scholarships-and-internships-to-apply-for-in-october-2026-1791380527</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="Q33" s="16" t="inlineStr">
         <is>
           <t>Means-based scholarship for first-year professional/open-degree students, 2026-27 cycle (applications close 31 October 2026). Included as Employment News-type central scholarship coverage; the specific EN issue placement was not directly verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GRID-INDIA "Vidyut Pragya" Specialised Internship in Power System Simulation Studies 2026-27</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Grid Controller of India Limited (GRID-INDIA), a Government of India enterprise under the Ministry of Power</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Full-time B.E./B.Tech/B.Sc.(Engg)/IDD in Electrical / Electrical (Power) / Electrical &amp; Electronics / Power Systems Engineering, with at least 65% or equivalent CGPA</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>All categories (SC/ST/PwBD marks relaxation up to pass marks)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>18 to 32 years as on 06/11/2026</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-27 (six-month internship, extendable by three months)</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Stipend Rs.50,000 per month (all-inclusive); 15 interns across NLDC/RLDC centres</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Online application 22/10/2026 to 06/11/2026</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>grid-india.in</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>https://grid-india.in ; https://dailysarkarijobs.com/grid-india-vidyut-pragya-internship-2026/</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Advertisement Ref. No. 2026_27/Internship/01 dated 21/10/2026. INFERRED from Employment News's normal coverage of central/PSU internships and apprenticeships (not directly seen in an EN issue); facts verified against the GRID-INDIA advertisement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DRDO Paid Internship 2026 (DRDE Gwalior)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Defence Research and Development Establishment (DRDE), DRDO, Ministry of Defence</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>M.Sc. or equivalent (3rd/4th semester) or B.Tech (7th/8th semester) in Biological Sciences, Chemical Sciences or Engineering, with at least 75% or CGPA 7.5</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>All categories</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Below 28 years as on 14/11/2026</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-27</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Stipend Rs.5,000 per month (Rs.30,000 in all for six months)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Apply by 14/11/2026 (by email); internship commences 01/01/2027</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>drdo.gov.in</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>https://www.educationtimes.com/news/drdo-internship-2026-apply-by-november-14-for-30000-stipend-check-eligibility-and-selection-process/articleshow/135066756.cms ; https://drdo.gov.in</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Reported 19-20 October 2026. INFERRED from Employment News's normal coverage of DRDO internship/apprenticeship notices (not directly seen in an EN issue).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>UGC National Eligibility Test (UGC-NET) December 2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>National Testing Agency (NTA), on behalf of the University Grants Commission (UGC)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Master's degree or equivalent with at least 55% marks (50% for reserved categories); final-year Master's students also eligible</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>All categories (category-wise fee)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Boys and girls</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No age limit for Assistant Professor; JRF upper age limit as per UGC norms (up to 30 years)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Twice-yearly (December 2026 session)</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Eligibility test for JRF, Assistant Professor and PhD admission; fee Rs.1,150 (General), Rs.600 (EWS/OBC-NCL), Rs.325 (SC/ST/PwD/third gender)</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Application 08/10/2026 to 28/10/2026 (late fee to 31/10/2026); exam 14-19/12/2026</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>ugcnet.nta.nic.in</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>https://ugcnet.nta.nic.in ; https://competition.careers360.com/articles/ugc-net-2026</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>New cycle (December 2026) of an exam Employment News has already logged for June 2025. INFERRED from its normal coverage (not directly seen in an EN issue); facts verified against NTA/aggregator pages.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(magazines): append RGIPT PhD 2026-27 entry
</commit_message>
<xml_diff>
--- a/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
+++ b/career-magazines/EmploymentNews_Log_Apr2025-Sep2026.xlsx
@@ -162,7 +162,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -256,6 +256,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -689,7 +692,7 @@
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Compiled 25 October 2026 | updated 25 October 2026 with the 1-25 October 2026 scrape</t>
+          <t>Compiled 26 October 2026 | updated automatically on each scheduled refresh. Sections: scholarships &amp; fellowships, internships, admissions / entrance exams (government job recruitment excluded).</t>
         </is>
       </c>
     </row>
@@ -733,8 +736,6 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="17"/>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17" ht="15" customHeight="1" s="17">
       <c r="B17" s="20" t="inlineStr">
         <is>
@@ -807,7 +808,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="17">
       <c r="B23" s="26" t="inlineStr">
         <is>
@@ -822,9 +822,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B9:D10"/>
+    <mergeCell ref="B11:D12"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="B13:D14"/>
-    <mergeCell ref="B11:D12"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q36"/>
+  <dimension ref="A1:Q37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="16" min="1" max="1"/>
@@ -3663,257 +3663,344 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>GRID-INDIA "Vidyut Pragya" Specialised Internship in Power System Simulation Studies 2026-27</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>Grid Controller of India Limited (GRID-INDIA), a Government of India enterprise under the Ministry of Power</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Full-time B.E./B.Tech/B.Sc.(Engg)/IDD in Electrical / Electrical (Power) / Electrical &amp; Electronics / Power Systems Engineering, with at least 65% or equivalent CGPA</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>All categories (SC/ST/PwBD marks relaxation up to pass marks)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="16" t="inlineStr">
         <is>
           <t>18 to 32 years as on 06/11/2026</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="16" t="inlineStr">
         <is>
           <t>2026-27 (six-month internship, extendable by three months)</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="K34" s="16" t="inlineStr">
         <is>
           <t>Stipend Rs.50,000 per month (all-inclusive); 15 interns across NLDC/RLDC centres</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="L34" s="16" t="inlineStr">
         <is>
           <t>Online application 22/10/2026 to 06/11/2026</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="M34" s="16" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="N34" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="O34" s="16" t="inlineStr">
         <is>
           <t>grid-india.in</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="P34" s="16" t="inlineStr">
         <is>
           <t>https://grid-india.in ; https://dailysarkarijobs.com/grid-india-vidyut-pragya-internship-2026/</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="Q34" s="16" t="inlineStr">
         <is>
           <t>Advertisement Ref. No. 2026_27/Internship/01 dated 21/10/2026. INFERRED from Employment News's normal coverage of central/PSU internships and apprenticeships (not directly seen in an EN issue); facts verified against the GRID-INDIA advertisement.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>DRDO Paid Internship 2026 (DRDE Gwalior)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="16" t="inlineStr">
         <is>
           <t>Defence Research and Development Establishment (DRDE), DRDO, Ministry of Defence</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>M.Sc. or equivalent (3rd/4th semester) or B.Tech (7th/8th semester) in Biological Sciences, Chemical Sciences or Engineering, with at least 75% or CGPA 7.5</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>All categories</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="16" t="inlineStr">
         <is>
           <t>Below 28 years as on 14/11/2026</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="16" t="inlineStr">
         <is>
           <t>2026-27</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="K35" s="16" t="inlineStr">
         <is>
           <t>Stipend Rs.5,000 per month (Rs.30,000 in all for six months)</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="L35" s="16" t="inlineStr">
         <is>
           <t>Apply by 14/11/2026 (by email); internship commences 01/01/2027</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="M35" s="16" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="N35" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="O35" s="16" t="inlineStr">
         <is>
           <t>drdo.gov.in</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" s="16" t="inlineStr">
         <is>
           <t>https://www.educationtimes.com/news/drdo-internship-2026-apply-by-november-14-for-30000-stipend-check-eligibility-and-selection-process/articleshow/135066756.cms ; https://drdo.gov.in</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
+      <c r="Q35" s="16" t="inlineStr">
         <is>
           <t>Reported 19-20 October 2026. INFERRED from Employment News's normal coverage of DRDO internship/apprenticeship notices (not directly seen in an EN issue).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Admission / Entrance Exam</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
         <is>
           <t>UGC National Eligibility Test (UGC-NET) December 2026</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>National Testing Agency (NTA), on behalf of the University Grants Commission (UGC)</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Master's degree or equivalent with at least 55% marks (50% for reserved categories); final-year Master's students also eligible</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>All categories (category-wise fee)</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="16" t="inlineStr">
         <is>
           <t>Boys and girls</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="16" t="inlineStr">
         <is>
           <t>Not applicable</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="16" t="inlineStr">
         <is>
           <t>No age limit for Assistant Professor; JRF upper age limit as per UGC norms (up to 30 years)</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="16" t="inlineStr">
         <is>
           <t>Twice-yearly (December 2026 session)</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="K36" s="16" t="inlineStr">
         <is>
           <t>Eligibility test for JRF, Assistant Professor and PhD admission; fee Rs.1,150 (General), Rs.600 (EWS/OBC-NCL), Rs.325 (SC/ST/PwD/third gender)</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="16" t="inlineStr">
         <is>
           <t>Application 08/10/2026 to 28/10/2026 (late fee to 31/10/2026); exam 14-19/12/2026</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M36" s="16" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N36" s="16" t="inlineStr">
         <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="O36" s="16" t="inlineStr">
         <is>
           <t>ugcnet.nta.nic.in</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" s="16" t="inlineStr">
         <is>
           <t>https://ugcnet.nta.nic.in ; https://competition.careers360.com/articles/ugc-net-2026</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="Q36" s="16" t="inlineStr">
         <is>
           <t>New cycle (December 2026) of an exam Employment News has already logged for June 2025. INFERRED from its normal coverage (not directly seen in an EN issue); facts verified against NTA/aggregator pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B37" s="32" t="inlineStr">
+        <is>
+          <t>Admission / Entrance Exam</t>
+        </is>
+      </c>
+      <c r="C37" s="32" t="inlineStr">
+        <is>
+          <t>Ph.D. Admissions 2026-27 (Even Semester) at RGIPT Jais, Bengaluru and Sivasagar campuses</t>
+        </is>
+      </c>
+      <c r="D37" s="32" t="inlineStr">
+        <is>
+          <t>Rajiv Gandhi Institute of Petroleum Technology (RGIPT), Jais, Amethi - an Institute of National Importance under the Ministry of Petroleum and Natural Gas</t>
+        </is>
+      </c>
+      <c r="E37" s="32" t="inlineStr">
+        <is>
+          <t>M.Tech/M.E. (60% or 6.0 CPI), M.Sc (60-65%), or a 4-year B.Tech/B.Sc (75% or 7.5 CPI) in engineering, sciences, humanities or management disciplines listed in Annexure-I</t>
+        </is>
+      </c>
+      <c r="F37" s="32" t="inlineStr">
+        <is>
+          <t>All categories (Government of India reservation norms; SC/ST get 5% / 0.5 CPI relaxation in the qualifying degree)</t>
+        </is>
+      </c>
+      <c r="G37" s="32" t="inlineStr">
+        <is>
+          <t>Boys and girls (women, SC/ST and PwD pay the lower application fee)</t>
+        </is>
+      </c>
+      <c r="H37" s="32" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="I37" s="32" t="inlineStr">
+        <is>
+          <t>No age limit prescribed in the admission notice</t>
+        </is>
+      </c>
+      <c r="J37" s="32" t="inlineStr">
+        <is>
+          <t>Even Semester, Academic Session 2026-27</t>
+        </is>
+      </c>
+      <c r="K37" s="32" t="inlineStr">
+        <is>
+          <t>Institute Assistantship (JRF) of Rs 37,000 per month with upgradation to SRF as per institute norms; 72 institute assistantships across departments; application fee Rs 1,200 plus GST (Rs 600 plus GST for SC/ST/PwD and women)</t>
+        </is>
+      </c>
+      <c r="L37" s="32" t="inlineStr">
+        <is>
+          <t>Online portal 16.10.2026 to 26.11.2026; shortlist notified 30.11.2026; written test/interview 11-12.12.2026; offers 15.12.2026; registration 28.12.2026; classes from 29.12.2026</t>
+        </is>
+      </c>
+      <c r="M37" s="32" t="inlineStr">
+        <is>
+          <t>Open now</t>
+        </is>
+      </c>
+      <c r="N37" s="32" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="O37" s="32" t="inlineStr">
+        <is>
+          <t>www.rgipt.ac.in</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>https://www.rgipt.ac.in/PhD-Admission-2026-27/ ; https://employmentnews.gov.in/newemp/MoreContentS.aspx?n=WebAdvertisement</t>
+        </is>
+      </c>
+      <c r="Q37" s="32" t="inlineStr">
+        <is>
+          <t>Listed as an Employment News web advertisement in issue no 29 (17-23 October 2026) under Rajiv Gandhi Institute of Petroleum Technology, Ministry of Petroleum and Natural Gas; dates, stipend and fee verified from RGIPT's official PhD admission page</t>
         </is>
       </c>
     </row>

</xml_diff>